<commit_message>
Atualiza planilhas Jul/26, overrides de nivel e portal de metas.
Sincroniza NEs e acompanhamento de SAIs com julho conferido, inclui
overrides de nivel/pontos (103172 e 102874), indicadores SAM/SAIL e
o pacote metas-analista para a coordenacao e gerente.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/nes-definicao.xlsx
+++ b/data/nes-definicao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trten-my.sharepoint.com/personal/marielli_neves_thomsonreuters_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD2BBD68-5B0F-4AE3-9C10-D63462B18640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B940EB4-EC2C-4C30-8840-C85D0D7A9AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="59" activeTab="59" xr2:uid="{24F8D716-B721-47FD-91DB-BCBECDFEEC93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="60" activeTab="60" xr2:uid="{24F8D716-B721-47FD-91DB-BCBECDFEEC93}"/>
   </bookViews>
   <sheets>
     <sheet name="Janeiro 2024 - Escrita" sheetId="1" r:id="rId1"/>
@@ -73,8 +73,10 @@
     <sheet name="Maio 2026 - Importação" sheetId="63" r:id="rId58"/>
     <sheet name="Junho 2026 - Escrita" sheetId="64" r:id="rId59"/>
     <sheet name="Junho 2026 - Importação" sheetId="65" r:id="rId60"/>
-    <sheet name="NEs GRAVES" sheetId="56" r:id="rId61"/>
-    <sheet name="Graficos" sheetId="40" r:id="rId62"/>
+    <sheet name="Julho 2026 - Escrita" sheetId="66" r:id="rId61"/>
+    <sheet name="Julho 2026 - Importação" sheetId="67" r:id="rId62"/>
+    <sheet name="NEs GRAVES" sheetId="56" r:id="rId63"/>
+    <sheet name="Graficos" sheetId="40" r:id="rId64"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -145,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1958" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2027" uniqueCount="408">
   <si>
     <t>LEVANTAMENTO DE NEs COM DEFINIÇÃO DO MÓDULO ESCRITA FISCAL - VERSÃO DE JANEIRO/2024 (10.4A-01)</t>
   </si>
@@ -1186,6 +1188,54 @@
   </si>
   <si>
     <t>Definiu incorretamente considerando a data da competência do arquivo e não do pagamento e o exemplo não tratou a condição do cliente.</t>
+  </si>
+  <si>
+    <t>Bárbara T.</t>
+  </si>
+  <si>
+    <t>Não foi avaliado a opção "Gerar lançamento na conta cliente/fornecedor para parcelas pagas a vista".</t>
+  </si>
+  <si>
+    <t>Bárbara L.</t>
+  </si>
+  <si>
+    <t>Não foi definido corretamente a regra de importar de anos anteriores as informações de Outros dados DEFIS API.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Não foi tratado o informativo DIEF. Precisamos ainda continuar tratando? </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Não deveria ter definição.</t>
+    </r>
+  </si>
+  <si>
+    <t>Antiga.</t>
+  </si>
+  <si>
+    <t>Felipi F</t>
+  </si>
+  <si>
+    <t>Foi alterado o comportamento da versão de mercado da apuração dos impostos de SCP. Revisão feita sem conferir comportamento de todos os impostos.</t>
+  </si>
+  <si>
+    <t>Não foi tratado os impostos 18-ISS Retido e 26-INSS Retido</t>
+  </si>
+  <si>
+    <t>Não tratou a Declaração Mensal e Recibo através da publicação feita pelo Onvio Processos, quando a atividade for publicada pela DAS API Integra Contador.</t>
   </si>
   <si>
     <t>VERSÃO DE JANEIRO DE 2026</t>
@@ -1348,7 +1398,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1442,6 +1492,13 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="14">
@@ -1658,7 +1715,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="271">
+  <cellXfs count="279">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2150,19 +2207,31 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2178,6 +2247,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2209,6 +2281,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2753,15 +2828,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -3067,15 +3142,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -3191,9 +3266,9 @@
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="248"/>
-      <c r="E10" s="248"/>
-      <c r="F10" s="248"/>
+      <c r="D10" s="254"/>
+      <c r="E10" s="254"/>
+      <c r="F10" s="254"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7">
@@ -3333,15 +3408,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -3625,15 +3700,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -3702,9 +3777,9 @@
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="248"/>
-      <c r="E7" s="248"/>
-      <c r="F7" s="248"/>
+      <c r="D7" s="254"/>
+      <c r="E7" s="254"/>
+      <c r="F7" s="254"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7">
@@ -3842,15 +3917,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -4168,15 +4243,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -4241,9 +4316,9 @@
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="248"/>
-      <c r="E7" s="248"/>
-      <c r="F7" s="248"/>
+      <c r="D7" s="254"/>
+      <c r="E7" s="254"/>
+      <c r="F7" s="254"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7">
@@ -4378,15 +4453,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -4612,15 +4687,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -4723,9 +4798,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
+      <c r="D9" s="254"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -4848,15 +4923,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -5076,15 +5151,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -5175,9 +5250,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
+      <c r="D9" s="254"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -5298,15 +5373,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -5640,15 +5715,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -5738,11 +5813,11 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="248" t="s">
+      <c r="D8" s="254" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="248"/>
-      <c r="F8" s="248"/>
+      <c r="E8" s="254"/>
+      <c r="F8" s="254"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -5882,15 +5957,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -5983,9 +6058,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
+      <c r="D9" s="254"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -6107,15 +6182,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -6416,15 +6491,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -6535,9 +6610,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
+      <c r="D9" s="254"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -6667,14 +6742,14 @@
       <c r="C1" s="66" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="249" t="s">
+      <c r="E1" s="255" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="249"/>
-      <c r="H1" s="250" t="s">
+      <c r="F1" s="255"/>
+      <c r="H1" s="256" t="s">
         <v>109</v>
       </c>
-      <c r="I1" s="251"/>
+      <c r="I1" s="257"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="66"/>
@@ -6811,15 +6886,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -7010,16 +7085,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
-      <c r="H1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -7158,9 +7233,9 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
-      <c r="G9" s="248"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
+      <c r="G9" s="254"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
@@ -7292,15 +7367,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -7526,16 +7601,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
-      <c r="H1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -7686,9 +7761,9 @@
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="20"/>
-      <c r="E9" s="252"/>
-      <c r="F9" s="252"/>
-      <c r="G9" s="252"/>
+      <c r="E9" s="258"/>
+      <c r="F9" s="258"/>
+      <c r="G9" s="258"/>
       <c r="H9" s="110"/>
     </row>
     <row r="10" spans="1:8">
@@ -7813,15 +7888,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -8017,16 +8092,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
-      <c r="H1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -8183,9 +8258,9 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
-      <c r="G9" s="248"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
+      <c r="G9" s="254"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
@@ -8310,15 +8385,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -8614,15 +8689,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -8819,15 +8894,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -8934,9 +9009,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
+      <c r="D9" s="254"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -9053,15 +9128,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -9268,16 +9343,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="253"/>
-      <c r="C1" s="253"/>
-      <c r="D1" s="253"/>
-      <c r="E1" s="253"/>
-      <c r="F1" s="253"/>
-      <c r="G1" s="253"/>
-      <c r="H1" s="254"/>
+      <c r="B1" s="260"/>
+      <c r="C1" s="260"/>
+      <c r="D1" s="260"/>
+      <c r="E1" s="260"/>
+      <c r="F1" s="260"/>
+      <c r="G1" s="260"/>
+      <c r="H1" s="261"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -9436,9 +9511,9 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
-      <c r="G9" s="248"/>
+      <c r="E9" s="254"/>
+      <c r="F9" s="254"/>
+      <c r="G9" s="254"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
@@ -9563,15 +9638,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -9807,16 +9882,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
-      <c r="H1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -10041,15 +10116,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -10293,15 +10368,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -10357,9 +10432,9 @@
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="248"/>
-      <c r="E6" s="248"/>
-      <c r="F6" s="248"/>
+      <c r="D6" s="254"/>
+      <c r="E6" s="254"/>
+      <c r="F6" s="254"/>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7">
@@ -10474,15 +10549,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>178</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -10740,15 +10815,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -10984,15 +11059,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -11070,11 +11145,11 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="248" t="s">
+      <c r="D8" s="254" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="248"/>
-      <c r="F8" s="248"/>
+      <c r="E8" s="254"/>
+      <c r="F8" s="254"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -11212,15 +11287,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>206</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -11478,15 +11553,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -11690,15 +11765,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -11956,15 +12031,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -12194,15 +12269,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -12477,15 +12552,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -12701,15 +12776,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>249</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -13031,15 +13106,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -13255,12 +13330,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A1" s="262" t="s">
+      <c r="A1" s="269" t="s">
         <v>256</v>
       </c>
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
+      <c r="B1" s="269"/>
+      <c r="C1" s="269"/>
+      <c r="D1" s="269"/>
       <c r="E1" s="88"/>
       <c r="F1" s="88"/>
       <c r="G1" s="88"/>
@@ -13287,14 +13362,14 @@
       <c r="G2" s="94" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="259" t="s">
+      <c r="I2" s="266" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="259"/>
-      <c r="L2" s="260" t="s">
+      <c r="J2" s="266"/>
+      <c r="L2" s="267" t="s">
         <v>109</v>
       </c>
-      <c r="M2" s="261"/>
+      <c r="M2" s="268"/>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="67" t="s">
@@ -13764,12 +13839,12 @@
       </c>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="262" t="s">
+      <c r="A17" s="269" t="s">
         <v>278</v>
       </c>
-      <c r="B17" s="262"/>
-      <c r="C17" s="262"/>
-      <c r="D17" s="262"/>
+      <c r="B17" s="269"/>
+      <c r="C17" s="269"/>
+      <c r="D17" s="269"/>
       <c r="E17" s="88"/>
       <c r="F17" s="88"/>
       <c r="G17" s="88"/>
@@ -14146,12 +14221,12 @@
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="255">
+      <c r="A35" s="262">
         <v>2025</v>
       </c>
-      <c r="B35" s="255"/>
-      <c r="C35" s="255"/>
-      <c r="D35" s="255"/>
+      <c r="B35" s="262"/>
+      <c r="C35" s="262"/>
+      <c r="D35" s="262"/>
       <c r="E35" s="195"/>
     </row>
     <row r="36" spans="1:7">
@@ -14209,12 +14284,12 @@
       <c r="E39" s="188"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="256">
+      <c r="A40" s="263">
         <v>2026</v>
       </c>
-      <c r="B40" s="257"/>
-      <c r="C40" s="257"/>
-      <c r="D40" s="258"/>
+      <c r="B40" s="264"/>
+      <c r="C40" s="264"/>
+      <c r="D40" s="265"/>
       <c r="E40" s="67"/>
     </row>
     <row r="41" spans="1:7">
@@ -14295,15 +14370,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -14630,15 +14705,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -14882,15 +14957,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -15120,15 +15195,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>301</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -15393,15 +15468,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>304</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -15622,15 +15697,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>311</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
       <c r="H1" s="238"/>
     </row>
     <row r="2" spans="1:9">
@@ -15988,15 +16063,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -16180,13 +16255,13 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="246">
+      <c r="A18" s="270">
         <v>2026</v>
       </c>
-      <c r="B18" s="246"/>
-      <c r="C18" s="246"/>
-      <c r="D18" s="246"/>
-      <c r="E18" s="246"/>
+      <c r="B18" s="270"/>
+      <c r="C18" s="270"/>
+      <c r="D18" s="270"/>
+      <c r="E18" s="270"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181" t="s">
@@ -16255,15 +16330,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
@@ -16688,15 +16763,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>330</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -16857,11 +16932,11 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="246"/>
-      <c r="B18" s="246"/>
-      <c r="C18" s="246"/>
-      <c r="D18" s="246"/>
-      <c r="E18" s="246"/>
+      <c r="A18" s="270"/>
+      <c r="B18" s="270"/>
+      <c r="C18" s="270"/>
+      <c r="D18" s="270"/>
+      <c r="E18" s="270"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181"/>
@@ -16909,15 +16984,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
@@ -17317,15 +17392,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>336</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -17550,11 +17625,11 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="246"/>
-      <c r="B18" s="246"/>
-      <c r="C18" s="246"/>
-      <c r="D18" s="246"/>
-      <c r="E18" s="246"/>
+      <c r="A18" s="270"/>
+      <c r="B18" s="270"/>
+      <c r="C18" s="270"/>
+      <c r="D18" s="270"/>
+      <c r="E18" s="270"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181"/>
@@ -17608,15 +17683,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
@@ -17982,15 +18057,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -18090,9 +18165,9 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="248"/>
-      <c r="E8" s="248"/>
-      <c r="F8" s="248"/>
+      <c r="D8" s="254"/>
+      <c r="E8" s="254"/>
+      <c r="F8" s="254"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -18234,15 +18309,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="259" t="s">
         <v>336</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -18449,11 +18524,11 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="246"/>
-      <c r="B18" s="246"/>
-      <c r="C18" s="246"/>
-      <c r="D18" s="246"/>
-      <c r="E18" s="246"/>
+      <c r="A18" s="270"/>
+      <c r="B18" s="270"/>
+      <c r="C18" s="270"/>
+      <c r="D18" s="270"/>
+      <c r="E18" s="270"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181"/>
@@ -18493,6 +18568,629 @@
 </file>
 
 <file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B202DD86-BB6C-4F51-B631-F17769582108}">
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+    <col min="7" max="7" width="147.42578125" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="251" t="s">
+        <v>331</v>
+      </c>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="142" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="234" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="66" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="210">
+        <v>101154</v>
+      </c>
+      <c r="B4" s="210">
+        <v>98414</v>
+      </c>
+      <c r="C4" s="153">
+        <v>2025</v>
+      </c>
+      <c r="D4" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>347</v>
+      </c>
+      <c r="F4" s="153" t="s">
+        <v>152</v>
+      </c>
+      <c r="G4" s="239" t="s">
+        <v>348</v>
+      </c>
+      <c r="H4" s="67" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="154">
+        <v>101342</v>
+      </c>
+      <c r="B5" s="154">
+        <v>90909</v>
+      </c>
+      <c r="C5" s="153">
+        <v>2024</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>349</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>350</v>
+      </c>
+      <c r="H5" s="67" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="216" customFormat="1">
+      <c r="A6" s="249">
+        <v>102176</v>
+      </c>
+      <c r="B6" s="214">
+        <v>89666</v>
+      </c>
+      <c r="C6" s="246">
+        <v>2024</v>
+      </c>
+      <c r="D6" s="247" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="247" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="247" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="248" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="158" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="27" customFormat="1">
+      <c r="A7" s="149">
+        <v>102310</v>
+      </c>
+      <c r="B7" s="149">
+        <v>98112</v>
+      </c>
+      <c r="C7" s="141">
+        <v>2025</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>349</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="250" t="s">
+        <v>351</v>
+      </c>
+      <c r="H7" s="137" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="53" customFormat="1">
+      <c r="A8" s="243">
+        <v>102589</v>
+      </c>
+      <c r="B8" s="243">
+        <v>8456</v>
+      </c>
+      <c r="C8" s="244">
+        <v>2008</v>
+      </c>
+      <c r="D8" s="54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="55" t="s">
+        <v>352</v>
+      </c>
+      <c r="H8" s="245" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="154">
+        <v>102677</v>
+      </c>
+      <c r="B9" s="154">
+        <v>101293</v>
+      </c>
+      <c r="C9" s="150">
+        <v>2026</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>353</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>354</v>
+      </c>
+      <c r="H9" s="67" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="154">
+        <v>102889</v>
+      </c>
+      <c r="B10" s="154">
+        <v>98663</v>
+      </c>
+      <c r="C10" s="150">
+        <v>2025</v>
+      </c>
+      <c r="D10" s="152" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="152" t="s">
+        <v>209</v>
+      </c>
+      <c r="F10" s="152" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="241" t="s">
+        <v>355</v>
+      </c>
+      <c r="H10" s="67" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="154">
+        <v>103129</v>
+      </c>
+      <c r="B11" s="154">
+        <v>95815</v>
+      </c>
+      <c r="C11" s="150">
+        <v>2025</v>
+      </c>
+      <c r="D11" s="152" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="152" t="s">
+        <v>353</v>
+      </c>
+      <c r="F11" s="152" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="241" t="s">
+        <v>356</v>
+      </c>
+      <c r="H11" s="67" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="154"/>
+      <c r="B12" s="154"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="152"/>
+      <c r="E12" s="152"/>
+      <c r="F12" s="152"/>
+      <c r="G12" s="236"/>
+      <c r="H12" s="67"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="154"/>
+      <c r="B13" s="154"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="67"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="154"/>
+      <c r="B14" s="154"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="67"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1">
+        <v>32</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1">
+        <v>8</v>
+      </c>
+      <c r="D18" s="7">
+        <f>C18/C17</f>
+        <v>0.25</v>
+      </c>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1">
+        <v>5</v>
+      </c>
+      <c r="D19" s="7">
+        <f>C19/C17</f>
+        <v>0.15625</v>
+      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" display="101154" xr:uid="{E292FE64-21F9-41F3-B3C0-3EC95BE234FD}"/>
+    <hyperlink ref="B4" r:id="rId2" display="98414" xr:uid="{91C40594-3D2C-411E-A953-AD7345131777}"/>
+    <hyperlink ref="A5" r:id="rId3" display="101342" xr:uid="{FDBD44B3-A289-42AA-903C-A8A11E4B531A}"/>
+    <hyperlink ref="B5" r:id="rId4" display="90909" xr:uid="{52FD083A-B9CF-4762-BA2E-B872FBCBC21D}"/>
+    <hyperlink ref="A6" r:id="rId5" display="102176" xr:uid="{DF95508B-C28B-4575-BC7F-2109EBDB3364}"/>
+    <hyperlink ref="B6" r:id="rId6" display="89666" xr:uid="{75132F4D-9FB9-4B09-8BB7-E61F70B6A2B6}"/>
+    <hyperlink ref="A7" r:id="rId7" display="102310" xr:uid="{602F93D5-445D-4233-8260-9F7043E62D70}"/>
+    <hyperlink ref="B7" r:id="rId8" display="98112" xr:uid="{4475E7EB-09E7-4000-BFB0-441B13D0AB17}"/>
+    <hyperlink ref="A8" r:id="rId9" display="102589" xr:uid="{7CE0B803-C3C3-4133-AFAC-506DF480F8EF}"/>
+    <hyperlink ref="B8" r:id="rId10" display="8456" xr:uid="{76EFE028-B477-4EF1-BE0B-CBE5DDD8085D}"/>
+    <hyperlink ref="A9" r:id="rId11" display="102677" xr:uid="{8DA4F18C-6294-4315-9A55-71C591631182}"/>
+    <hyperlink ref="B9" r:id="rId12" display="101293" xr:uid="{FBC2DB54-BCC0-46DB-8619-6DD37769635B}"/>
+    <hyperlink ref="A10" r:id="rId13" display="102889" xr:uid="{1CAA2A11-40F8-4385-8763-E4BB7F4E3C78}"/>
+    <hyperlink ref="A11" r:id="rId14" display="103129" xr:uid="{57326F75-DFB1-4E87-A6DC-A24372FC81B3}"/>
+    <hyperlink ref="B11" r:id="rId15" display="95815" xr:uid="{08DE0E2C-E15B-4873-9E93-73001FF09D19}"/>
+    <hyperlink ref="B10" r:id="rId16" display="98663" xr:uid="{3296255E-43F5-4539-A603-A37012BE69FC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796B6919-CC0B-4776-83CC-64066396AC10}">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+    <col min="7" max="7" width="147.42578125" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="251" t="s">
+        <v>331</v>
+      </c>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="142" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="234" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="66" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="210">
+        <v>102683</v>
+      </c>
+      <c r="B4" s="210">
+        <v>102651</v>
+      </c>
+      <c r="C4" s="153">
+        <v>2026</v>
+      </c>
+      <c r="D4" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="153" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="239" t="s">
+        <v>81</v>
+      </c>
+      <c r="H4" s="67" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="216" customFormat="1">
+      <c r="A5" s="214">
+        <v>102320</v>
+      </c>
+      <c r="B5" s="214" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="246"/>
+      <c r="D5" s="247"/>
+      <c r="E5" s="247"/>
+      <c r="F5" s="247"/>
+      <c r="G5" s="248"/>
+      <c r="H5" s="158" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="210"/>
+      <c r="B6" s="154"/>
+      <c r="C6" s="153"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="67"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="154"/>
+      <c r="B7" s="154"/>
+      <c r="C7" s="150"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="67"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="154"/>
+      <c r="B8" s="154"/>
+      <c r="C8" s="150"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="67"/>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="154"/>
+      <c r="B9" s="154"/>
+      <c r="C9" s="150"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="67"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="154"/>
+      <c r="B10" s="154"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="67"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="154"/>
+      <c r="B11" s="154"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="67"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="7">
+        <f>C15/C14</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="7">
+        <f>C16/C14</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" display="102683" xr:uid="{5A276D18-98C4-4849-B328-FF883744028E}"/>
+    <hyperlink ref="B4" r:id="rId2" display="102651" xr:uid="{A8B88415-69E6-4082-AFC1-78431DB27CCE}"/>
+    <hyperlink ref="A5" r:id="rId3" display="102320" xr:uid="{18D95C0D-3796-4C03-B8B7-340A28C24E4E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA6F61C5-A8B9-4671-A779-2313F63F9507}">
   <dimension ref="A1:K45"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18509,31 +19207,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="216" customFormat="1">
-      <c r="A1" s="269" t="s">
-        <v>347</v>
-      </c>
-      <c r="B1" s="269"/>
-      <c r="C1" s="269"/>
-      <c r="D1" s="269"/>
-      <c r="E1" s="269"/>
-      <c r="F1" s="269"/>
-      <c r="G1" s="269"/>
-      <c r="H1" s="269"/>
-      <c r="I1" s="269"/>
+      <c r="A1" s="277" t="s">
+        <v>357</v>
+      </c>
+      <c r="B1" s="277"/>
+      <c r="C1" s="277"/>
+      <c r="D1" s="277"/>
+      <c r="E1" s="277"/>
+      <c r="F1" s="277"/>
+      <c r="G1" s="277"/>
+      <c r="H1" s="277"/>
+      <c r="I1" s="277"/>
       <c r="J1" s="158"/>
     </row>
     <row r="2" spans="1:10" s="216" customFormat="1">
-      <c r="A2" s="267" t="s">
+      <c r="A2" s="275" t="s">
         <v>256</v>
       </c>
-      <c r="B2" s="267"/>
-      <c r="C2" s="267"/>
-      <c r="D2" s="267"/>
-      <c r="E2" s="267"/>
-      <c r="F2" s="267"/>
-      <c r="G2" s="267"/>
-      <c r="H2" s="267"/>
-      <c r="I2" s="267"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
       <c r="J2" s="158"/>
     </row>
     <row r="3" spans="1:10" s="216" customFormat="1">
@@ -18556,16 +19254,16 @@
         <v>6</v>
       </c>
       <c r="G3" s="217" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="H3" s="217" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="I3" s="159" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="J3" s="159" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="216" customFormat="1">
@@ -18588,7 +19286,7 @@
         <v>152</v>
       </c>
       <c r="G4" s="158" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="H4" s="158" t="s">
         <v>112</v>
@@ -18621,31 +19319,31 @@
       <c r="J6" s="67"/>
     </row>
     <row r="7" spans="1:10" s="216" customFormat="1">
-      <c r="A7" s="269" t="s">
-        <v>353</v>
-      </c>
-      <c r="B7" s="269"/>
-      <c r="C7" s="269"/>
-      <c r="D7" s="269"/>
-      <c r="E7" s="269"/>
-      <c r="F7" s="269"/>
-      <c r="G7" s="269"/>
-      <c r="H7" s="269"/>
-      <c r="I7" s="269"/>
+      <c r="A7" s="277" t="s">
+        <v>363</v>
+      </c>
+      <c r="B7" s="277"/>
+      <c r="C7" s="277"/>
+      <c r="D7" s="277"/>
+      <c r="E7" s="277"/>
+      <c r="F7" s="277"/>
+      <c r="G7" s="277"/>
+      <c r="H7" s="277"/>
+      <c r="I7" s="277"/>
       <c r="J7" s="158"/>
     </row>
     <row r="8" spans="1:10" s="216" customFormat="1">
-      <c r="A8" s="267" t="s">
+      <c r="A8" s="275" t="s">
         <v>256</v>
       </c>
-      <c r="B8" s="267"/>
-      <c r="C8" s="267"/>
-      <c r="D8" s="267"/>
-      <c r="E8" s="267"/>
-      <c r="F8" s="267"/>
-      <c r="G8" s="267"/>
-      <c r="H8" s="267"/>
-      <c r="I8" s="267"/>
+      <c r="B8" s="275"/>
+      <c r="C8" s="275"/>
+      <c r="D8" s="275"/>
+      <c r="E8" s="275"/>
+      <c r="F8" s="275"/>
+      <c r="G8" s="275"/>
+      <c r="H8" s="275"/>
+      <c r="I8" s="275"/>
       <c r="J8" s="158"/>
     </row>
     <row r="9" spans="1:10" s="216" customFormat="1">
@@ -18668,16 +19366,16 @@
         <v>6</v>
       </c>
       <c r="G9" s="217" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="H9" s="217" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="I9" s="159" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="J9" s="159" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="45.75">
@@ -18700,16 +19398,16 @@
         <v>33</v>
       </c>
       <c r="G10" s="67" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="H10" s="67" t="s">
         <v>112</v>
       </c>
       <c r="I10" s="162" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="J10" s="161" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="30.75">
@@ -18732,16 +19430,16 @@
         <v>33</v>
       </c>
       <c r="G11" s="67" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
       <c r="H11" s="67" t="s">
         <v>112</v>
       </c>
       <c r="I11" s="163" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="J11" s="160" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="216" customFormat="1">
@@ -18764,13 +19462,13 @@
         <v>35</v>
       </c>
       <c r="G12" s="158" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="H12" s="158" t="s">
         <v>112</v>
       </c>
       <c r="I12" s="158" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="J12" s="225"/>
     </row>
@@ -18794,13 +19492,13 @@
         <v>19</v>
       </c>
       <c r="G13" s="158" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
       <c r="H13" s="158" t="s">
         <v>112</v>
       </c>
       <c r="I13" s="158" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="J13" s="158"/>
     </row>
@@ -18824,13 +19522,13 @@
         <v>33</v>
       </c>
       <c r="G14" s="158" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
       <c r="H14" s="158" t="s">
         <v>112</v>
       </c>
       <c r="I14" s="158" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="J14" s="158"/>
     </row>
@@ -18854,28 +19552,28 @@
         <v>33</v>
       </c>
       <c r="G15" s="158" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="H15" s="158" t="s">
         <v>112</v>
       </c>
       <c r="I15" s="158" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="J15" s="158"/>
     </row>
     <row r="16" spans="1:10" s="216" customFormat="1">
-      <c r="A16" s="267" t="s">
+      <c r="A16" s="275" t="s">
         <v>278</v>
       </c>
-      <c r="B16" s="267"/>
-      <c r="C16" s="267"/>
-      <c r="D16" s="267"/>
-      <c r="E16" s="267"/>
-      <c r="F16" s="267"/>
-      <c r="G16" s="267"/>
-      <c r="H16" s="267"/>
-      <c r="I16" s="267"/>
+      <c r="B16" s="275"/>
+      <c r="C16" s="275"/>
+      <c r="D16" s="275"/>
+      <c r="E16" s="275"/>
+      <c r="F16" s="275"/>
+      <c r="G16" s="275"/>
+      <c r="H16" s="275"/>
+      <c r="I16" s="275"/>
       <c r="J16" s="158"/>
     </row>
     <row r="17" spans="1:11" s="216" customFormat="1">
@@ -18898,13 +19596,13 @@
         <v>28</v>
       </c>
       <c r="G17" s="158" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="H17" s="158" t="s">
         <v>112</v>
       </c>
       <c r="I17" s="158" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="J17" s="158"/>
     </row>
@@ -18933,31 +19631,31 @@
       <c r="J19" s="67"/>
     </row>
     <row r="20" spans="1:11" s="216" customFormat="1">
-      <c r="A20" s="263" t="s">
-        <v>366</v>
-      </c>
-      <c r="B20" s="263"/>
-      <c r="C20" s="263"/>
-      <c r="D20" s="263"/>
-      <c r="E20" s="263"/>
-      <c r="F20" s="263"/>
-      <c r="G20" s="263"/>
-      <c r="H20" s="263"/>
-      <c r="I20" s="263"/>
+      <c r="A20" s="271" t="s">
+        <v>376</v>
+      </c>
+      <c r="B20" s="271"/>
+      <c r="C20" s="271"/>
+      <c r="D20" s="271"/>
+      <c r="E20" s="271"/>
+      <c r="F20" s="271"/>
+      <c r="G20" s="271"/>
+      <c r="H20" s="271"/>
+      <c r="I20" s="271"/>
       <c r="J20" s="158"/>
     </row>
     <row r="21" spans="1:11" s="216" customFormat="1">
-      <c r="A21" s="267" t="s">
+      <c r="A21" s="275" t="s">
         <v>256</v>
       </c>
-      <c r="B21" s="267"/>
-      <c r="C21" s="267"/>
-      <c r="D21" s="267"/>
-      <c r="E21" s="267"/>
-      <c r="F21" s="267"/>
-      <c r="G21" s="267"/>
-      <c r="H21" s="267"/>
-      <c r="I21" s="267"/>
+      <c r="B21" s="275"/>
+      <c r="C21" s="275"/>
+      <c r="D21" s="275"/>
+      <c r="E21" s="275"/>
+      <c r="F21" s="275"/>
+      <c r="G21" s="275"/>
+      <c r="H21" s="275"/>
+      <c r="I21" s="275"/>
       <c r="J21" s="158"/>
     </row>
     <row r="22" spans="1:11" s="216" customFormat="1">
@@ -18980,16 +19678,16 @@
         <v>6</v>
       </c>
       <c r="G22" s="224" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="H22" s="224" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="I22" s="164" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="J22" s="164" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="173" customFormat="1">
@@ -19012,17 +19710,17 @@
         <v>10</v>
       </c>
       <c r="G23" s="172" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="H23" s="172" t="s">
         <v>151</v>
       </c>
       <c r="I23" s="172"/>
       <c r="J23" s="172" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="K23" s="173" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -19045,14 +19743,14 @@
         <v>35</v>
       </c>
       <c r="G24" s="67" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="H24" s="67" t="s">
         <v>151</v>
       </c>
       <c r="I24" s="67"/>
       <c r="J24" s="67" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -19075,14 +19773,14 @@
         <v>33</v>
       </c>
       <c r="G25" s="67" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="H25" s="67" t="s">
         <v>151</v>
       </c>
       <c r="I25" s="67"/>
       <c r="J25" s="67" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="216" customFormat="1">
@@ -19105,13 +19803,13 @@
         <v>35</v>
       </c>
       <c r="G26" s="158" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
       <c r="H26" s="158" t="s">
         <v>112</v>
       </c>
       <c r="I26" s="158" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="J26" s="158"/>
     </row>
@@ -19135,7 +19833,7 @@
         <v>35</v>
       </c>
       <c r="G27" s="158" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="H27" s="158" t="s">
         <v>112</v>
@@ -19144,31 +19842,31 @@
       <c r="J27" s="158"/>
     </row>
     <row r="28" spans="1:11" s="216" customFormat="1">
-      <c r="A28" s="263" t="s">
-        <v>376</v>
-      </c>
-      <c r="B28" s="263"/>
-      <c r="C28" s="263"/>
-      <c r="D28" s="263"/>
-      <c r="E28" s="263"/>
-      <c r="F28" s="263"/>
-      <c r="G28" s="263"/>
-      <c r="H28" s="263"/>
-      <c r="I28" s="263"/>
+      <c r="A28" s="271" t="s">
+        <v>386</v>
+      </c>
+      <c r="B28" s="271"/>
+      <c r="C28" s="271"/>
+      <c r="D28" s="271"/>
+      <c r="E28" s="271"/>
+      <c r="F28" s="271"/>
+      <c r="G28" s="271"/>
+      <c r="H28" s="271"/>
+      <c r="I28" s="271"/>
       <c r="J28" s="207"/>
     </row>
     <row r="29" spans="1:11" s="216" customFormat="1">
-      <c r="A29" s="267" t="s">
+      <c r="A29" s="275" t="s">
         <v>256</v>
       </c>
-      <c r="B29" s="267"/>
-      <c r="C29" s="267"/>
-      <c r="D29" s="267"/>
-      <c r="E29" s="267"/>
-      <c r="F29" s="267"/>
-      <c r="G29" s="267"/>
-      <c r="H29" s="267"/>
-      <c r="I29" s="267"/>
+      <c r="B29" s="275"/>
+      <c r="C29" s="275"/>
+      <c r="D29" s="275"/>
+      <c r="E29" s="275"/>
+      <c r="F29" s="275"/>
+      <c r="G29" s="275"/>
+      <c r="H29" s="275"/>
+      <c r="I29" s="275"/>
       <c r="J29" s="158"/>
     </row>
     <row r="30" spans="1:11" s="216" customFormat="1">
@@ -19191,16 +19889,16 @@
         <v>6</v>
       </c>
       <c r="G30" s="217" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="H30" s="217" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="I30" s="159" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="J30" s="159" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -19227,10 +19925,10 @@
         <v>151</v>
       </c>
       <c r="I31" s="67" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
       <c r="J31" s="67" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
     </row>
     <row r="32" spans="1:11" s="216" customFormat="1">
@@ -19260,17 +19958,17 @@
       <c r="J32" s="158"/>
     </row>
     <row r="33" spans="1:10" s="216" customFormat="1">
-      <c r="A33" s="267" t="s">
+      <c r="A33" s="275" t="s">
         <v>278</v>
       </c>
-      <c r="B33" s="267"/>
-      <c r="C33" s="267"/>
-      <c r="D33" s="267"/>
-      <c r="E33" s="267"/>
-      <c r="F33" s="267"/>
-      <c r="G33" s="267"/>
-      <c r="H33" s="267"/>
-      <c r="I33" s="267"/>
+      <c r="B33" s="275"/>
+      <c r="C33" s="275"/>
+      <c r="D33" s="275"/>
+      <c r="E33" s="275"/>
+      <c r="F33" s="275"/>
+      <c r="G33" s="275"/>
+      <c r="H33" s="275"/>
+      <c r="I33" s="275"/>
       <c r="J33" s="207"/>
     </row>
     <row r="34" spans="1:10" s="216" customFormat="1">
@@ -19326,31 +20024,31 @@
       <c r="J35" s="158"/>
     </row>
     <row r="36" spans="1:10" s="216" customFormat="1">
-      <c r="A36" s="263" t="s">
-        <v>379</v>
-      </c>
-      <c r="B36" s="263"/>
-      <c r="C36" s="263"/>
-      <c r="D36" s="263"/>
-      <c r="E36" s="263"/>
-      <c r="F36" s="263"/>
-      <c r="G36" s="263"/>
-      <c r="H36" s="263"/>
-      <c r="I36" s="264"/>
+      <c r="A36" s="271" t="s">
+        <v>389</v>
+      </c>
+      <c r="B36" s="271"/>
+      <c r="C36" s="271"/>
+      <c r="D36" s="271"/>
+      <c r="E36" s="271"/>
+      <c r="F36" s="271"/>
+      <c r="G36" s="271"/>
+      <c r="H36" s="271"/>
+      <c r="I36" s="272"/>
       <c r="J36" s="158"/>
     </row>
     <row r="37" spans="1:10" s="216" customFormat="1">
-      <c r="A37" s="267" t="s">
+      <c r="A37" s="275" t="s">
         <v>256</v>
       </c>
-      <c r="B37" s="267"/>
-      <c r="C37" s="267"/>
-      <c r="D37" s="267"/>
-      <c r="E37" s="267"/>
-      <c r="F37" s="267"/>
-      <c r="G37" s="267"/>
-      <c r="H37" s="267"/>
-      <c r="I37" s="268"/>
+      <c r="B37" s="275"/>
+      <c r="C37" s="275"/>
+      <c r="D37" s="275"/>
+      <c r="E37" s="275"/>
+      <c r="F37" s="275"/>
+      <c r="G37" s="275"/>
+      <c r="H37" s="275"/>
+      <c r="I37" s="276"/>
       <c r="J37" s="158"/>
     </row>
     <row r="38" spans="1:10" s="216" customFormat="1">
@@ -19373,13 +20071,13 @@
         <v>6</v>
       </c>
       <c r="G38" s="217" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="H38" s="217" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="I38" s="223" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="J38" s="158"/>
     </row>
@@ -19410,30 +20108,30 @@
       <c r="J39" s="158"/>
     </row>
     <row r="40" spans="1:10" s="216" customFormat="1">
-      <c r="A40" s="263" t="s">
-        <v>380</v>
-      </c>
-      <c r="B40" s="263"/>
-      <c r="C40" s="263"/>
-      <c r="D40" s="263"/>
-      <c r="E40" s="263"/>
-      <c r="F40" s="263"/>
-      <c r="G40" s="263"/>
-      <c r="H40" s="263"/>
-      <c r="I40" s="264"/>
+      <c r="A40" s="271" t="s">
+        <v>390</v>
+      </c>
+      <c r="B40" s="271"/>
+      <c r="C40" s="271"/>
+      <c r="D40" s="271"/>
+      <c r="E40" s="271"/>
+      <c r="F40" s="271"/>
+      <c r="G40" s="271"/>
+      <c r="H40" s="271"/>
+      <c r="I40" s="272"/>
     </row>
     <row r="41" spans="1:10" s="216" customFormat="1">
-      <c r="A41" s="265" t="s">
+      <c r="A41" s="273" t="s">
         <v>256</v>
       </c>
-      <c r="B41" s="265"/>
-      <c r="C41" s="265"/>
-      <c r="D41" s="265"/>
-      <c r="E41" s="265"/>
-      <c r="F41" s="265"/>
-      <c r="G41" s="265"/>
-      <c r="H41" s="265"/>
-      <c r="I41" s="266"/>
+      <c r="B41" s="273"/>
+      <c r="C41" s="273"/>
+      <c r="D41" s="273"/>
+      <c r="E41" s="273"/>
+      <c r="F41" s="273"/>
+      <c r="G41" s="273"/>
+      <c r="H41" s="273"/>
+      <c r="I41" s="274"/>
     </row>
     <row r="42" spans="1:10" s="216" customFormat="1">
       <c r="A42" s="217" t="s">
@@ -19455,13 +20153,13 @@
         <v>6</v>
       </c>
       <c r="G42" s="217" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="H42" s="217" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="I42" s="159" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -19605,7 +20303,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E31C6E68-DA8C-48AA-B9DD-835E99E5F9F6}">
   <dimension ref="A5:N76"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19623,7 +20321,7 @@
   <sheetData>
     <row r="5" spans="1:10" ht="37.5" customHeight="1">
       <c r="A5" s="94" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
       <c r="B5" s="66" t="s">
         <v>105</v>
@@ -19632,7 +20330,7 @@
         <v>106</v>
       </c>
       <c r="D5" s="93" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="E5" s="69" t="s">
         <v>259</v>
@@ -19641,7 +20339,7 @@
         <v>260</v>
       </c>
       <c r="G5" s="94" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -20013,7 +20711,7 @@
     </row>
     <row r="21" spans="1:10" ht="30.75">
       <c r="A21" s="94" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
       <c r="B21" s="66" t="s">
         <v>105</v>
@@ -20022,7 +20720,7 @@
         <v>106</v>
       </c>
       <c r="D21" s="93" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="E21" s="69" t="s">
         <v>259</v>
@@ -20031,7 +20729,7 @@
         <v>260</v>
       </c>
       <c r="G21" s="94" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -20355,43 +21053,43 @@
       </c>
     </row>
     <row r="44" spans="1:14">
-      <c r="A44" s="250" t="s">
-        <v>387</v>
-      </c>
-      <c r="B44" s="270"/>
-      <c r="C44" s="270"/>
-      <c r="D44" s="270"/>
-      <c r="E44" s="270"/>
-      <c r="F44" s="270"/>
-      <c r="G44" s="270"/>
-      <c r="H44" s="270"/>
-      <c r="I44" s="270"/>
-      <c r="J44" s="270"/>
-      <c r="K44" s="270"/>
-      <c r="L44" s="270"/>
-      <c r="M44" s="251"/>
+      <c r="A44" s="256" t="s">
+        <v>397</v>
+      </c>
+      <c r="B44" s="278"/>
+      <c r="C44" s="278"/>
+      <c r="D44" s="278"/>
+      <c r="E44" s="278"/>
+      <c r="F44" s="278"/>
+      <c r="G44" s="278"/>
+      <c r="H44" s="278"/>
+      <c r="I44" s="278"/>
+      <c r="J44" s="278"/>
+      <c r="K44" s="278"/>
+      <c r="L44" s="278"/>
+      <c r="M44" s="257"/>
       <c r="N44" s="66" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="67" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
       <c r="B45" s="227">
         <v>46023</v>
       </c>
       <c r="C45" s="67" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
       <c r="D45" s="227">
         <v>46082</v>
       </c>
       <c r="E45" s="67" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="F45" s="67" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="G45" s="227">
         <v>46174</v>
@@ -20400,19 +21098,19 @@
         <v>46204</v>
       </c>
       <c r="I45" s="67" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="J45" s="67" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="K45" s="67" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="L45" s="227">
         <v>46327</v>
       </c>
       <c r="M45" s="67" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="N45" s="74"/>
     </row>
@@ -20640,22 +21338,22 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="67" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
       <c r="B56" s="227">
         <v>46023</v>
       </c>
       <c r="C56" s="67" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
       <c r="D56" s="227">
         <v>46082</v>
       </c>
       <c r="E56" s="67" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="F56" s="67" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="G56" s="227">
         <v>46174</v>
@@ -20664,22 +21362,22 @@
         <v>46204</v>
       </c>
       <c r="I56" s="67" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="J56" s="67" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="K56" s="67" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="L56" s="227">
         <v>46327</v>
       </c>
       <c r="M56" s="67" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="N56" s="66" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -20816,14 +21514,14 @@
       </c>
     </row>
     <row r="66" spans="1:5">
-      <c r="A66" s="259" t="s">
+      <c r="A66" s="266" t="s">
         <v>108</v>
       </c>
-      <c r="B66" s="259"/>
-      <c r="D66" s="249" t="s">
+      <c r="B66" s="266"/>
+      <c r="D66" s="255" t="s">
         <v>109</v>
       </c>
-      <c r="E66" s="249"/>
+      <c r="E66" s="255"/>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="67" t="s">
@@ -20983,15 +21681,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -21324,15 +22022,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="245"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="253"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -21462,9 +22160,9 @@
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="248"/>
-      <c r="E10" s="248"/>
-      <c r="F10" s="248"/>
+      <c r="D10" s="254"/>
+      <c r="E10" s="254"/>
+      <c r="F10" s="254"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7">
@@ -21607,15 +22305,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="251" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>

</xml_diff>

<commit_message>
Inclui retornos NE, acomp. SAM/SAIL e corrige casamento de nomes na planilha.
Separa homonimas (Rafaela/Barbara), enriquece cache de metas, atualiza planilhas e indicadores de tempo/SS.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/nes-definicao.xlsx
+++ b/data/nes-definicao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trten-my.sharepoint.com/personal/marielli_neves_thomsonreuters_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B940EB4-EC2C-4C30-8840-C85D0D7A9AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{347A3526-9F7A-4CDA-8150-832512C73F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="60" activeTab="60" xr2:uid="{24F8D716-B721-47FD-91DB-BCBECDFEEC93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="63" activeTab="61" xr2:uid="{24F8D716-B721-47FD-91DB-BCBECDFEEC93}"/>
   </bookViews>
   <sheets>
     <sheet name="Janeiro 2024 - Escrita" sheetId="1" r:id="rId1"/>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2027" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2046" uniqueCount="409">
   <si>
     <t>LEVANTAMENTO DE NEs COM DEFINIÇÃO DO MÓDULO ESCRITA FISCAL - VERSÃO DE JANEIRO/2024 (10.4A-01)</t>
   </si>
@@ -1338,6 +1338,9 @@
   </si>
   <si>
     <t>VERSÃO DE JUNHO DE 2026</t>
+  </si>
+  <si>
+    <t>VERSÃO DE JULHO DE 2026</t>
   </si>
   <si>
     <t>Versão 2025</t>
@@ -1715,7 +1718,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="279">
+  <cellXfs count="284">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2225,6 +2228,36 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2235,15 +2268,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2268,9 +2292,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2298,16 +2319,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2828,15 +2846,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -3142,15 +3160,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -3266,9 +3284,9 @@
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="254"/>
-      <c r="E10" s="254"/>
-      <c r="F10" s="254"/>
+      <c r="D10" s="264"/>
+      <c r="E10" s="264"/>
+      <c r="F10" s="264"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7">
@@ -3408,15 +3426,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -3700,15 +3718,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -3777,9 +3795,9 @@
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="254"/>
-      <c r="E7" s="254"/>
-      <c r="F7" s="254"/>
+      <c r="D7" s="264"/>
+      <c r="E7" s="264"/>
+      <c r="F7" s="264"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7">
@@ -3917,15 +3935,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -4243,15 +4261,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -4316,9 +4334,9 @@
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="254"/>
-      <c r="E7" s="254"/>
-      <c r="F7" s="254"/>
+      <c r="D7" s="264"/>
+      <c r="E7" s="264"/>
+      <c r="F7" s="264"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7">
@@ -4453,15 +4471,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -4687,15 +4705,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -4798,9 +4816,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="254"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
+      <c r="D9" s="264"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -4923,15 +4941,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -5151,15 +5169,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -5250,9 +5268,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="254"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
+      <c r="D9" s="264"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -5373,15 +5391,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -5715,15 +5733,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -5813,11 +5831,11 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="254" t="s">
+      <c r="D8" s="264" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="254"/>
-      <c r="F8" s="254"/>
+      <c r="E8" s="264"/>
+      <c r="F8" s="264"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -5957,15 +5975,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -6058,9 +6076,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="254"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
+      <c r="D9" s="264"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -6182,15 +6200,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -6491,15 +6509,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -6610,9 +6628,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="254"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
+      <c r="D9" s="264"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -6742,14 +6760,14 @@
       <c r="C1" s="66" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="255" t="s">
+      <c r="E1" s="260" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="255"/>
+      <c r="F1" s="260"/>
       <c r="H1" s="256" t="s">
         <v>109</v>
       </c>
-      <c r="I1" s="257"/>
+      <c r="I1" s="258"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="66"/>
@@ -6886,15 +6904,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -7085,16 +7103,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -7233,9 +7251,9 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
-      <c r="G9" s="254"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
+      <c r="G9" s="264"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
@@ -7367,15 +7385,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -7601,16 +7619,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -7761,9 +7779,9 @@
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="20"/>
-      <c r="E9" s="258"/>
-      <c r="F9" s="258"/>
-      <c r="G9" s="258"/>
+      <c r="E9" s="265"/>
+      <c r="F9" s="265"/>
+      <c r="G9" s="265"/>
       <c r="H9" s="110"/>
     </row>
     <row r="10" spans="1:8">
@@ -7888,15 +7906,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -8092,16 +8110,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -8258,9 +8276,9 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
-      <c r="G9" s="254"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
+      <c r="G9" s="264"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
@@ -8385,15 +8403,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -8689,15 +8707,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -8894,15 +8912,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -9009,9 +9027,9 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="254"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
+      <c r="D9" s="264"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7">
@@ -9128,15 +9146,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -9343,16 +9361,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="260"/>
-      <c r="C1" s="260"/>
-      <c r="D1" s="260"/>
-      <c r="E1" s="260"/>
-      <c r="F1" s="260"/>
-      <c r="G1" s="260"/>
-      <c r="H1" s="261"/>
+      <c r="B1" s="267"/>
+      <c r="C1" s="267"/>
+      <c r="D1" s="267"/>
+      <c r="E1" s="267"/>
+      <c r="F1" s="267"/>
+      <c r="G1" s="267"/>
+      <c r="H1" s="268"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -9511,9 +9529,9 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="254"/>
-      <c r="F9" s="254"/>
-      <c r="G9" s="254"/>
+      <c r="E9" s="264"/>
+      <c r="F9" s="264"/>
+      <c r="G9" s="264"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
@@ -9638,15 +9656,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -9882,16 +9900,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -10116,15 +10134,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -10368,15 +10386,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -10432,9 +10450,9 @@
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="254"/>
-      <c r="E6" s="254"/>
-      <c r="F6" s="254"/>
+      <c r="D6" s="264"/>
+      <c r="E6" s="264"/>
+      <c r="F6" s="264"/>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7">
@@ -10549,15 +10567,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>178</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -10815,15 +10833,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -11059,15 +11077,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -11145,11 +11163,11 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="254" t="s">
+      <c r="D8" s="264" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="254"/>
-      <c r="F8" s="254"/>
+      <c r="E8" s="264"/>
+      <c r="F8" s="264"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -11287,15 +11305,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>206</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -11553,15 +11571,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -11765,15 +11783,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -12031,15 +12049,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -12269,15 +12287,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -12552,15 +12570,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -12776,15 +12794,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>249</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -13106,15 +13124,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -13330,12 +13348,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A1" s="269" t="s">
+      <c r="A1" s="275" t="s">
         <v>256</v>
       </c>
-      <c r="B1" s="269"/>
-      <c r="C1" s="269"/>
-      <c r="D1" s="269"/>
+      <c r="B1" s="275"/>
+      <c r="C1" s="275"/>
+      <c r="D1" s="275"/>
       <c r="E1" s="88"/>
       <c r="F1" s="88"/>
       <c r="G1" s="88"/>
@@ -13362,14 +13380,14 @@
       <c r="G2" s="94" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="266" t="s">
+      <c r="I2" s="259" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="266"/>
-      <c r="L2" s="267" t="s">
+      <c r="J2" s="259"/>
+      <c r="L2" s="273" t="s">
         <v>109</v>
       </c>
-      <c r="M2" s="268"/>
+      <c r="M2" s="274"/>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="67" t="s">
@@ -13839,12 +13857,12 @@
       </c>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="269" t="s">
+      <c r="A17" s="275" t="s">
         <v>278</v>
       </c>
-      <c r="B17" s="269"/>
-      <c r="C17" s="269"/>
-      <c r="D17" s="269"/>
+      <c r="B17" s="275"/>
+      <c r="C17" s="275"/>
+      <c r="D17" s="275"/>
       <c r="E17" s="88"/>
       <c r="F17" s="88"/>
       <c r="G17" s="88"/>
@@ -14221,12 +14239,12 @@
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="262">
+      <c r="A35" s="269">
         <v>2025</v>
       </c>
-      <c r="B35" s="262"/>
-      <c r="C35" s="262"/>
-      <c r="D35" s="262"/>
+      <c r="B35" s="269"/>
+      <c r="C35" s="269"/>
+      <c r="D35" s="269"/>
       <c r="E35" s="195"/>
     </row>
     <row r="36" spans="1:7">
@@ -14284,12 +14302,12 @@
       <c r="E39" s="188"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="263">
+      <c r="A40" s="270">
         <v>2026</v>
       </c>
-      <c r="B40" s="264"/>
-      <c r="C40" s="264"/>
-      <c r="D40" s="265"/>
+      <c r="B40" s="271"/>
+      <c r="C40" s="271"/>
+      <c r="D40" s="272"/>
       <c r="E40" s="67"/>
     </row>
     <row r="41" spans="1:7">
@@ -14370,15 +14388,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -14705,15 +14723,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -14957,15 +14975,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -15195,15 +15213,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>301</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -15468,15 +15486,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>304</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -15697,15 +15715,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>311</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
       <c r="H1" s="238"/>
     </row>
     <row r="2" spans="1:9">
@@ -16063,15 +16081,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -16255,13 +16273,13 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="270">
+      <c r="A18" s="276">
         <v>2026</v>
       </c>
-      <c r="B18" s="270"/>
-      <c r="C18" s="270"/>
-      <c r="D18" s="270"/>
-      <c r="E18" s="270"/>
+      <c r="B18" s="276"/>
+      <c r="C18" s="276"/>
+      <c r="D18" s="276"/>
+      <c r="E18" s="276"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181" t="s">
@@ -16330,15 +16348,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
@@ -16763,15 +16781,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>330</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -16932,11 +16950,11 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="270"/>
-      <c r="B18" s="270"/>
-      <c r="C18" s="270"/>
-      <c r="D18" s="270"/>
-      <c r="E18" s="270"/>
+      <c r="A18" s="276"/>
+      <c r="B18" s="276"/>
+      <c r="C18" s="276"/>
+      <c r="D18" s="276"/>
+      <c r="E18" s="276"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181"/>
@@ -16984,15 +17002,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
@@ -17392,15 +17410,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>336</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -17625,11 +17643,11 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="270"/>
-      <c r="B18" s="270"/>
-      <c r="C18" s="270"/>
-      <c r="D18" s="270"/>
-      <c r="E18" s="270"/>
+      <c r="A18" s="276"/>
+      <c r="B18" s="276"/>
+      <c r="C18" s="276"/>
+      <c r="D18" s="276"/>
+      <c r="E18" s="276"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181"/>
@@ -17683,15 +17701,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
@@ -18057,15 +18075,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -18165,9 +18183,9 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="254"/>
-      <c r="E8" s="254"/>
-      <c r="F8" s="254"/>
+      <c r="D8" s="264"/>
+      <c r="E8" s="264"/>
+      <c r="F8" s="264"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -18309,15 +18327,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="266" t="s">
         <v>336</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5"/>
@@ -18524,11 +18542,11 @@
       <c r="G14" s="1"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="270"/>
-      <c r="B18" s="270"/>
-      <c r="C18" s="270"/>
-      <c r="D18" s="270"/>
-      <c r="E18" s="270"/>
+      <c r="A18" s="276"/>
+      <c r="B18" s="276"/>
+      <c r="C18" s="276"/>
+      <c r="D18" s="276"/>
+      <c r="E18" s="276"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="181"/>
@@ -18583,15 +18601,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -18680,29 +18698,29 @@
         <v>151</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="216" customFormat="1">
-      <c r="A6" s="249">
+    <row r="6" spans="1:8" s="53" customFormat="1">
+      <c r="A6" s="254">
         <v>102176</v>
       </c>
-      <c r="B6" s="214">
+      <c r="B6" s="243">
         <v>89666</v>
       </c>
-      <c r="C6" s="246">
+      <c r="C6" s="255">
         <v>2024</v>
       </c>
-      <c r="D6" s="247" t="s">
+      <c r="D6" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="247" t="s">
+      <c r="E6" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="247" t="s">
+      <c r="F6" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="248" t="s">
+      <c r="G6" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="158" t="s">
+      <c r="H6" s="245" t="s">
         <v>112</v>
       </c>
     </row>
@@ -18967,15 +18985,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1"/>
@@ -19012,29 +19030,29 @@
         <v>283</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="210">
+    <row r="4" spans="1:8" s="216" customFormat="1">
+      <c r="A4" s="249">
         <v>102683</v>
       </c>
-      <c r="B4" s="210">
+      <c r="B4" s="249">
         <v>102651</v>
       </c>
-      <c r="C4" s="153">
+      <c r="C4" s="246">
         <v>2026</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D4" s="251" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="49" t="s">
+      <c r="E4" s="251" t="s">
         <v>59</v>
       </c>
-      <c r="F4" s="153" t="s">
+      <c r="F4" s="246" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="239" t="s">
+      <c r="G4" s="252" t="s">
         <v>81</v>
       </c>
-      <c r="H4" s="67" t="s">
+      <c r="H4" s="158" t="s">
         <v>112</v>
       </c>
     </row>
@@ -19192,7 +19210,7 @@
 
 <file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA6F61C5-A8B9-4671-A779-2313F63F9507}">
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -19207,31 +19225,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="216" customFormat="1">
-      <c r="A1" s="277" t="s">
+      <c r="A1" s="281" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="277"/>
-      <c r="C1" s="277"/>
-      <c r="D1" s="277"/>
-      <c r="E1" s="277"/>
-      <c r="F1" s="277"/>
-      <c r="G1" s="277"/>
-      <c r="H1" s="277"/>
-      <c r="I1" s="277"/>
+      <c r="B1" s="281"/>
+      <c r="C1" s="281"/>
+      <c r="D1" s="281"/>
+      <c r="E1" s="281"/>
+      <c r="F1" s="281"/>
+      <c r="G1" s="281"/>
+      <c r="H1" s="281"/>
+      <c r="I1" s="281"/>
       <c r="J1" s="158"/>
     </row>
     <row r="2" spans="1:10" s="216" customFormat="1">
-      <c r="A2" s="275" t="s">
+      <c r="A2" s="282" t="s">
         <v>256</v>
       </c>
-      <c r="B2" s="275"/>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
+      <c r="B2" s="282"/>
+      <c r="C2" s="282"/>
+      <c r="D2" s="282"/>
+      <c r="E2" s="282"/>
+      <c r="F2" s="282"/>
+      <c r="G2" s="282"/>
+      <c r="H2" s="282"/>
+      <c r="I2" s="282"/>
       <c r="J2" s="158"/>
     </row>
     <row r="3" spans="1:10" s="216" customFormat="1">
@@ -19319,31 +19337,31 @@
       <c r="J6" s="67"/>
     </row>
     <row r="7" spans="1:10" s="216" customFormat="1">
-      <c r="A7" s="277" t="s">
+      <c r="A7" s="281" t="s">
         <v>363</v>
       </c>
-      <c r="B7" s="277"/>
-      <c r="C7" s="277"/>
-      <c r="D7" s="277"/>
-      <c r="E7" s="277"/>
-      <c r="F7" s="277"/>
-      <c r="G7" s="277"/>
-      <c r="H7" s="277"/>
-      <c r="I7" s="277"/>
+      <c r="B7" s="281"/>
+      <c r="C7" s="281"/>
+      <c r="D7" s="281"/>
+      <c r="E7" s="281"/>
+      <c r="F7" s="281"/>
+      <c r="G7" s="281"/>
+      <c r="H7" s="281"/>
+      <c r="I7" s="281"/>
       <c r="J7" s="158"/>
     </row>
     <row r="8" spans="1:10" s="216" customFormat="1">
-      <c r="A8" s="275" t="s">
+      <c r="A8" s="282" t="s">
         <v>256</v>
       </c>
-      <c r="B8" s="275"/>
-      <c r="C8" s="275"/>
-      <c r="D8" s="275"/>
-      <c r="E8" s="275"/>
-      <c r="F8" s="275"/>
-      <c r="G8" s="275"/>
-      <c r="H8" s="275"/>
-      <c r="I8" s="275"/>
+      <c r="B8" s="282"/>
+      <c r="C8" s="282"/>
+      <c r="D8" s="282"/>
+      <c r="E8" s="282"/>
+      <c r="F8" s="282"/>
+      <c r="G8" s="282"/>
+      <c r="H8" s="282"/>
+      <c r="I8" s="282"/>
       <c r="J8" s="158"/>
     </row>
     <row r="9" spans="1:10" s="216" customFormat="1">
@@ -19563,17 +19581,17 @@
       <c r="J15" s="158"/>
     </row>
     <row r="16" spans="1:10" s="216" customFormat="1">
-      <c r="A16" s="275" t="s">
+      <c r="A16" s="282" t="s">
         <v>278</v>
       </c>
-      <c r="B16" s="275"/>
-      <c r="C16" s="275"/>
-      <c r="D16" s="275"/>
-      <c r="E16" s="275"/>
-      <c r="F16" s="275"/>
-      <c r="G16" s="275"/>
-      <c r="H16" s="275"/>
-      <c r="I16" s="275"/>
+      <c r="B16" s="282"/>
+      <c r="C16" s="282"/>
+      <c r="D16" s="282"/>
+      <c r="E16" s="282"/>
+      <c r="F16" s="282"/>
+      <c r="G16" s="282"/>
+      <c r="H16" s="282"/>
+      <c r="I16" s="282"/>
       <c r="J16" s="158"/>
     </row>
     <row r="17" spans="1:11" s="216" customFormat="1">
@@ -19631,31 +19649,31 @@
       <c r="J19" s="67"/>
     </row>
     <row r="20" spans="1:11" s="216" customFormat="1">
-      <c r="A20" s="271" t="s">
+      <c r="A20" s="277" t="s">
         <v>376</v>
       </c>
-      <c r="B20" s="271"/>
-      <c r="C20" s="271"/>
-      <c r="D20" s="271"/>
-      <c r="E20" s="271"/>
-      <c r="F20" s="271"/>
-      <c r="G20" s="271"/>
-      <c r="H20" s="271"/>
-      <c r="I20" s="271"/>
+      <c r="B20" s="277"/>
+      <c r="C20" s="277"/>
+      <c r="D20" s="277"/>
+      <c r="E20" s="277"/>
+      <c r="F20" s="277"/>
+      <c r="G20" s="277"/>
+      <c r="H20" s="277"/>
+      <c r="I20" s="277"/>
       <c r="J20" s="158"/>
     </row>
     <row r="21" spans="1:11" s="216" customFormat="1">
-      <c r="A21" s="275" t="s">
+      <c r="A21" s="282" t="s">
         <v>256</v>
       </c>
-      <c r="B21" s="275"/>
-      <c r="C21" s="275"/>
-      <c r="D21" s="275"/>
-      <c r="E21" s="275"/>
-      <c r="F21" s="275"/>
-      <c r="G21" s="275"/>
-      <c r="H21" s="275"/>
-      <c r="I21" s="275"/>
+      <c r="B21" s="282"/>
+      <c r="C21" s="282"/>
+      <c r="D21" s="282"/>
+      <c r="E21" s="282"/>
+      <c r="F21" s="282"/>
+      <c r="G21" s="282"/>
+      <c r="H21" s="282"/>
+      <c r="I21" s="282"/>
       <c r="J21" s="158"/>
     </row>
     <row r="22" spans="1:11" s="216" customFormat="1">
@@ -19842,31 +19860,31 @@
       <c r="J27" s="158"/>
     </row>
     <row r="28" spans="1:11" s="216" customFormat="1">
-      <c r="A28" s="271" t="s">
+      <c r="A28" s="277" t="s">
         <v>386</v>
       </c>
-      <c r="B28" s="271"/>
-      <c r="C28" s="271"/>
-      <c r="D28" s="271"/>
-      <c r="E28" s="271"/>
-      <c r="F28" s="271"/>
-      <c r="G28" s="271"/>
-      <c r="H28" s="271"/>
-      <c r="I28" s="271"/>
+      <c r="B28" s="277"/>
+      <c r="C28" s="277"/>
+      <c r="D28" s="277"/>
+      <c r="E28" s="277"/>
+      <c r="F28" s="277"/>
+      <c r="G28" s="277"/>
+      <c r="H28" s="277"/>
+      <c r="I28" s="277"/>
       <c r="J28" s="207"/>
     </row>
     <row r="29" spans="1:11" s="216" customFormat="1">
-      <c r="A29" s="275" t="s">
+      <c r="A29" s="282" t="s">
         <v>256</v>
       </c>
-      <c r="B29" s="275"/>
-      <c r="C29" s="275"/>
-      <c r="D29" s="275"/>
-      <c r="E29" s="275"/>
-      <c r="F29" s="275"/>
-      <c r="G29" s="275"/>
-      <c r="H29" s="275"/>
-      <c r="I29" s="275"/>
+      <c r="B29" s="282"/>
+      <c r="C29" s="282"/>
+      <c r="D29" s="282"/>
+      <c r="E29" s="282"/>
+      <c r="F29" s="282"/>
+      <c r="G29" s="282"/>
+      <c r="H29" s="282"/>
+      <c r="I29" s="282"/>
       <c r="J29" s="158"/>
     </row>
     <row r="30" spans="1:11" s="216" customFormat="1">
@@ -19958,17 +19976,17 @@
       <c r="J32" s="158"/>
     </row>
     <row r="33" spans="1:10" s="216" customFormat="1">
-      <c r="A33" s="275" t="s">
+      <c r="A33" s="282" t="s">
         <v>278</v>
       </c>
-      <c r="B33" s="275"/>
-      <c r="C33" s="275"/>
-      <c r="D33" s="275"/>
-      <c r="E33" s="275"/>
-      <c r="F33" s="275"/>
-      <c r="G33" s="275"/>
-      <c r="H33" s="275"/>
-      <c r="I33" s="275"/>
+      <c r="B33" s="282"/>
+      <c r="C33" s="282"/>
+      <c r="D33" s="282"/>
+      <c r="E33" s="282"/>
+      <c r="F33" s="282"/>
+      <c r="G33" s="282"/>
+      <c r="H33" s="282"/>
+      <c r="I33" s="282"/>
       <c r="J33" s="207"/>
     </row>
     <row r="34" spans="1:10" s="216" customFormat="1">
@@ -20024,31 +20042,31 @@
       <c r="J35" s="158"/>
     </row>
     <row r="36" spans="1:10" s="216" customFormat="1">
-      <c r="A36" s="271" t="s">
+      <c r="A36" s="277" t="s">
         <v>389</v>
       </c>
-      <c r="B36" s="271"/>
-      <c r="C36" s="271"/>
-      <c r="D36" s="271"/>
-      <c r="E36" s="271"/>
-      <c r="F36" s="271"/>
-      <c r="G36" s="271"/>
-      <c r="H36" s="271"/>
-      <c r="I36" s="272"/>
+      <c r="B36" s="277"/>
+      <c r="C36" s="277"/>
+      <c r="D36" s="277"/>
+      <c r="E36" s="277"/>
+      <c r="F36" s="277"/>
+      <c r="G36" s="277"/>
+      <c r="H36" s="277"/>
+      <c r="I36" s="278"/>
       <c r="J36" s="158"/>
     </row>
     <row r="37" spans="1:10" s="216" customFormat="1">
-      <c r="A37" s="275" t="s">
+      <c r="A37" s="282" t="s">
         <v>256</v>
       </c>
-      <c r="B37" s="275"/>
-      <c r="C37" s="275"/>
-      <c r="D37" s="275"/>
-      <c r="E37" s="275"/>
-      <c r="F37" s="275"/>
-      <c r="G37" s="275"/>
-      <c r="H37" s="275"/>
-      <c r="I37" s="276"/>
+      <c r="B37" s="282"/>
+      <c r="C37" s="282"/>
+      <c r="D37" s="282"/>
+      <c r="E37" s="282"/>
+      <c r="F37" s="282"/>
+      <c r="G37" s="282"/>
+      <c r="H37" s="282"/>
+      <c r="I37" s="283"/>
       <c r="J37" s="158"/>
     </row>
     <row r="38" spans="1:10" s="216" customFormat="1">
@@ -20108,30 +20126,30 @@
       <c r="J39" s="158"/>
     </row>
     <row r="40" spans="1:10" s="216" customFormat="1">
-      <c r="A40" s="271" t="s">
+      <c r="A40" s="277" t="s">
         <v>390</v>
       </c>
-      <c r="B40" s="271"/>
-      <c r="C40" s="271"/>
-      <c r="D40" s="271"/>
-      <c r="E40" s="271"/>
-      <c r="F40" s="271"/>
-      <c r="G40" s="271"/>
-      <c r="H40" s="271"/>
-      <c r="I40" s="272"/>
+      <c r="B40" s="277"/>
+      <c r="C40" s="277"/>
+      <c r="D40" s="277"/>
+      <c r="E40" s="277"/>
+      <c r="F40" s="277"/>
+      <c r="G40" s="277"/>
+      <c r="H40" s="277"/>
+      <c r="I40" s="278"/>
     </row>
     <row r="41" spans="1:10" s="216" customFormat="1">
-      <c r="A41" s="273" t="s">
+      <c r="A41" s="279" t="s">
         <v>256</v>
       </c>
-      <c r="B41" s="273"/>
-      <c r="C41" s="273"/>
-      <c r="D41" s="273"/>
-      <c r="E41" s="273"/>
-      <c r="F41" s="273"/>
-      <c r="G41" s="273"/>
-      <c r="H41" s="273"/>
-      <c r="I41" s="274"/>
+      <c r="B41" s="279"/>
+      <c r="C41" s="279"/>
+      <c r="D41" s="279"/>
+      <c r="E41" s="279"/>
+      <c r="F41" s="279"/>
+      <c r="G41" s="279"/>
+      <c r="H41" s="279"/>
+      <c r="I41" s="280"/>
     </row>
     <row r="42" spans="1:10" s="216" customFormat="1">
       <c r="A42" s="217" t="s">
@@ -20175,10 +20193,10 @@
       <c r="D43" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="E43" s="49" t="s">
+      <c r="E43" s="253" t="s">
         <v>312</v>
       </c>
-      <c r="F43" s="49" t="s">
+      <c r="F43" s="253" t="s">
         <v>33</v>
       </c>
       <c r="G43" s="95"/>
@@ -20200,10 +20218,10 @@
       <c r="D44" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E44" s="148" t="s">
         <v>209</v>
       </c>
-      <c r="F44" s="19" t="s">
+      <c r="F44" s="148" t="s">
         <v>33</v>
       </c>
       <c r="G44" s="67"/>
@@ -20237,8 +20255,115 @@
       </c>
       <c r="I45" s="158"/>
     </row>
+    <row r="46" spans="1:10">
+      <c r="A46" s="277" t="s">
+        <v>391</v>
+      </c>
+      <c r="B46" s="277"/>
+      <c r="C46" s="277"/>
+      <c r="D46" s="277"/>
+      <c r="E46" s="277"/>
+      <c r="F46" s="277"/>
+      <c r="G46" s="277"/>
+      <c r="H46" s="277"/>
+      <c r="I46" s="278"/>
+    </row>
+    <row r="47" spans="1:10">
+      <c r="A47" s="279" t="s">
+        <v>256</v>
+      </c>
+      <c r="B47" s="279"/>
+      <c r="C47" s="279"/>
+      <c r="D47" s="279"/>
+      <c r="E47" s="279"/>
+      <c r="F47" s="279"/>
+      <c r="G47" s="279"/>
+      <c r="H47" s="279"/>
+      <c r="I47" s="280"/>
+    </row>
+    <row r="48" spans="1:10">
+      <c r="A48" s="217" t="s">
+        <v>1</v>
+      </c>
+      <c r="B48" s="217" t="s">
+        <v>2</v>
+      </c>
+      <c r="C48" s="217" t="s">
+        <v>3</v>
+      </c>
+      <c r="D48" s="217" t="s">
+        <v>4</v>
+      </c>
+      <c r="E48" s="217" t="s">
+        <v>5</v>
+      </c>
+      <c r="F48" s="217" t="s">
+        <v>6</v>
+      </c>
+      <c r="G48" s="217" t="s">
+        <v>358</v>
+      </c>
+      <c r="H48" s="217" t="s">
+        <v>359</v>
+      </c>
+      <c r="I48" s="159" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="210">
+        <v>103098</v>
+      </c>
+      <c r="B49" s="210">
+        <v>99223</v>
+      </c>
+      <c r="C49" s="49">
+        <v>2026</v>
+      </c>
+      <c r="D49" s="49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" s="253" t="s">
+        <v>52</v>
+      </c>
+      <c r="F49" s="253" t="s">
+        <v>35</v>
+      </c>
+      <c r="G49" s="95"/>
+      <c r="H49" s="95" t="s">
+        <v>112</v>
+      </c>
+      <c r="I49" s="95"/>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="154">
+        <v>102736</v>
+      </c>
+      <c r="B50" s="154">
+        <v>101305</v>
+      </c>
+      <c r="C50" s="19">
+        <v>2026</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" s="148" t="s">
+        <v>52</v>
+      </c>
+      <c r="F50" s="148" t="s">
+        <v>35</v>
+      </c>
+      <c r="G50" s="67"/>
+      <c r="H50" s="67" t="s">
+        <v>112</v>
+      </c>
+      <c r="I50" s="67"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
+    <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A47:I47"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A20:I20"/>
@@ -20297,9 +20422,13 @@
     <hyperlink ref="B44" r:id="rId40" display="101855" xr:uid="{F24D0885-CF3F-4830-922C-668AAF5157C7}"/>
     <hyperlink ref="A45" r:id="rId41" display="101966" xr:uid="{2A769D8A-8C48-4EB2-B959-001B3E58F86A}"/>
     <hyperlink ref="B45" r:id="rId42" display="101487" xr:uid="{99E08F43-ABD4-42DC-94C0-906EB61565B3}"/>
+    <hyperlink ref="A49" r:id="rId43" display="103098" xr:uid="{911BADEB-C889-4274-A15D-5BDBD39F7FD3}"/>
+    <hyperlink ref="A50" r:id="rId44" display="102736" xr:uid="{ACF783D0-CC61-4E5E-BE48-5D62A781EB28}"/>
+    <hyperlink ref="B49" r:id="rId45" display="99223" xr:uid="{3BDF64AE-F713-47D3-87D7-13ED227C56FB}"/>
+    <hyperlink ref="B50" r:id="rId46" display="101305" xr:uid="{609F30ED-48BC-4D47-8271-32F62B41172B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId43"/>
+  <legacyDrawing r:id="rId47"/>
 </worksheet>
 </file>
 
@@ -20321,7 +20450,7 @@
   <sheetData>
     <row r="5" spans="1:10" ht="37.5" customHeight="1">
       <c r="A5" s="94" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B5" s="66" t="s">
         <v>105</v>
@@ -20330,7 +20459,7 @@
         <v>106</v>
       </c>
       <c r="D5" s="93" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E5" s="69" t="s">
         <v>259</v>
@@ -20339,7 +20468,7 @@
         <v>260</v>
       </c>
       <c r="G5" s="94" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -20711,7 +20840,7 @@
     </row>
     <row r="21" spans="1:10" ht="30.75">
       <c r="A21" s="94" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B21" s="66" t="s">
         <v>105</v>
@@ -20720,7 +20849,7 @@
         <v>106</v>
       </c>
       <c r="D21" s="93" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E21" s="69" t="s">
         <v>259</v>
@@ -20729,7 +20858,7 @@
         <v>260</v>
       </c>
       <c r="G21" s="94" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -21054,42 +21183,42 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="256" t="s">
-        <v>397</v>
-      </c>
-      <c r="B44" s="278"/>
-      <c r="C44" s="278"/>
-      <c r="D44" s="278"/>
-      <c r="E44" s="278"/>
-      <c r="F44" s="278"/>
-      <c r="G44" s="278"/>
-      <c r="H44" s="278"/>
-      <c r="I44" s="278"/>
-      <c r="J44" s="278"/>
-      <c r="K44" s="278"/>
-      <c r="L44" s="278"/>
-      <c r="M44" s="257"/>
+        <v>398</v>
+      </c>
+      <c r="B44" s="257"/>
+      <c r="C44" s="257"/>
+      <c r="D44" s="257"/>
+      <c r="E44" s="257"/>
+      <c r="F44" s="257"/>
+      <c r="G44" s="257"/>
+      <c r="H44" s="257"/>
+      <c r="I44" s="257"/>
+      <c r="J44" s="257"/>
+      <c r="K44" s="257"/>
+      <c r="L44" s="257"/>
+      <c r="M44" s="258"/>
       <c r="N44" s="66" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="67" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B45" s="227">
         <v>46023</v>
       </c>
       <c r="C45" s="67" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D45" s="227">
         <v>46082</v>
       </c>
       <c r="E45" s="67" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F45" s="67" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G45" s="227">
         <v>46174</v>
@@ -21098,19 +21227,19 @@
         <v>46204</v>
       </c>
       <c r="I45" s="67" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J45" s="67" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K45" s="67" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="L45" s="227">
         <v>46327</v>
       </c>
       <c r="M45" s="67" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="N45" s="74"/>
     </row>
@@ -21176,7 +21305,9 @@
         <v>2</v>
       </c>
       <c r="G48" s="67"/>
-      <c r="H48" s="67"/>
+      <c r="H48" s="67">
+        <v>1</v>
+      </c>
       <c r="I48" s="67"/>
       <c r="J48" s="67"/>
       <c r="K48" s="67"/>
@@ -21184,7 +21315,7 @@
       <c r="M48" s="67"/>
       <c r="N48" s="74">
         <f>B48+C48+D48+E48+F48+G48+H48+I48+J48+K48+L48+M48</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -21224,7 +21355,9 @@
       <c r="G50" s="67">
         <v>1</v>
       </c>
-      <c r="H50" s="67"/>
+      <c r="H50" s="67">
+        <v>2</v>
+      </c>
       <c r="I50" s="67"/>
       <c r="J50" s="67"/>
       <c r="K50" s="67"/>
@@ -21232,7 +21365,7 @@
       <c r="M50" s="67"/>
       <c r="N50" s="74">
         <f>B50+C50+D50+E50+F50+G50+H50+I50+J50+K50+L50+M50</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -21276,7 +21409,9 @@
       <c r="G52" s="67">
         <v>1</v>
       </c>
-      <c r="H52" s="67"/>
+      <c r="H52" s="67">
+        <v>1</v>
+      </c>
       <c r="I52" s="67"/>
       <c r="J52" s="67"/>
       <c r="K52" s="67"/>
@@ -21284,7 +21419,7 @@
       <c r="M52" s="67"/>
       <c r="N52" s="74">
         <f>B52+C52+D52+E52+F52+G52+H52+I52+J52+K52+L52+M52</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -21299,7 +21434,9 @@
         <v>1</v>
       </c>
       <c r="G53" s="67"/>
-      <c r="H53" s="67"/>
+      <c r="H53" s="67">
+        <v>1</v>
+      </c>
       <c r="I53" s="67"/>
       <c r="J53" s="67"/>
       <c r="K53" s="67"/>
@@ -21307,7 +21444,7 @@
       <c r="M53" s="67"/>
       <c r="N53" s="74">
         <f>B53+C53+D53+E53+F53+G53+H53+I53+J53+K53+L53+M53</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -21338,22 +21475,22 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="67" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B56" s="227">
         <v>46023</v>
       </c>
       <c r="C56" s="67" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D56" s="227">
         <v>46082</v>
       </c>
       <c r="E56" s="67" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F56" s="67" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G56" s="227">
         <v>46174</v>
@@ -21362,22 +21499,22 @@
         <v>46204</v>
       </c>
       <c r="I56" s="67" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J56" s="67" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K56" s="67" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="L56" s="227">
         <v>46327</v>
       </c>
       <c r="M56" s="67" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="N56" s="66" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -21394,7 +21531,9 @@
       </c>
       <c r="F57" s="67"/>
       <c r="G57" s="67"/>
-      <c r="H57" s="67"/>
+      <c r="H57" s="67">
+        <v>1</v>
+      </c>
       <c r="I57" s="67"/>
       <c r="J57" s="67"/>
       <c r="K57" s="67"/>
@@ -21402,7 +21541,7 @@
       <c r="M57" s="67"/>
       <c r="N57" s="74">
         <f>B57+C57+D57+E57+F57+G57+H57+I57+J57+K57+L57+M57</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -21427,7 +21566,9 @@
       <c r="G58" s="67">
         <v>2</v>
       </c>
-      <c r="H58" s="67"/>
+      <c r="H58" s="67">
+        <v>2</v>
+      </c>
       <c r="I58" s="67"/>
       <c r="J58" s="67"/>
       <c r="K58" s="67"/>
@@ -21435,7 +21576,7 @@
       <c r="M58" s="67"/>
       <c r="N58" s="74">
         <f>B58+C58+D58+E58+F58+G58+H58+I58+J58+K58+L58+M58</f>
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -21452,7 +21593,9 @@
       <c r="G59" s="67">
         <v>2</v>
       </c>
-      <c r="H59" s="67"/>
+      <c r="H59" s="67">
+        <v>1</v>
+      </c>
       <c r="I59" s="67"/>
       <c r="J59" s="67"/>
       <c r="K59" s="67"/>
@@ -21460,7 +21603,7 @@
       <c r="M59" s="67"/>
       <c r="N59" s="74">
         <f>B59+C59+D59+E59+F59+G59+H59+I59+J59+K59+L59+M59</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -21475,7 +21618,9 @@
       <c r="E60" s="67"/>
       <c r="F60" s="67"/>
       <c r="G60" s="67"/>
-      <c r="H60" s="67"/>
+      <c r="H60" s="67">
+        <v>1</v>
+      </c>
       <c r="I60" s="67"/>
       <c r="J60" s="67"/>
       <c r="K60" s="67"/>
@@ -21483,7 +21628,7 @@
       <c r="M60" s="67"/>
       <c r="N60" s="74">
         <f>B60+C60+D60+E60+F60+G60+H60+I60+J60+K60+L60+M60</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -21514,14 +21659,14 @@
       </c>
     </row>
     <row r="66" spans="1:5">
-      <c r="A66" s="266" t="s">
+      <c r="A66" s="259" t="s">
         <v>108</v>
       </c>
-      <c r="B66" s="266"/>
-      <c r="D66" s="255" t="s">
+      <c r="B66" s="259"/>
+      <c r="D66" s="260" t="s">
         <v>109</v>
       </c>
-      <c r="E66" s="255"/>
+      <c r="E66" s="260"/>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="67" t="s">
@@ -21535,8 +21680,7 @@
         <v>152</v>
       </c>
       <c r="E67" s="67">
-        <f>N60</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -21544,8 +21688,7 @@
         <v>9</v>
       </c>
       <c r="B68" s="67">
-        <f>N50</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D68" s="67" t="s">
         <v>10</v>
@@ -21560,15 +21703,13 @@
         <v>265</v>
       </c>
       <c r="B69" s="67">
-        <f>N53</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D69" s="67" t="s">
         <v>19</v>
       </c>
       <c r="E69" s="67">
-        <f>N57</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -21576,15 +21717,13 @@
         <v>14</v>
       </c>
       <c r="B70" s="67">
-        <f>N48</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D70" s="67" t="s">
         <v>35</v>
       </c>
       <c r="E70" s="67">
-        <f>N58</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -21599,8 +21738,7 @@
         <v>189</v>
       </c>
       <c r="E71" s="67">
-        <f>N59</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -21626,15 +21764,14 @@
         <v>209</v>
       </c>
       <c r="B74" s="67">
-        <f>N52</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D74" s="67" t="s">
         <v>271</v>
       </c>
       <c r="E74" s="100">
         <f>E67+E68+E69+E70+E71</f>
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -21652,7 +21789,7 @@
       </c>
       <c r="B76" s="100">
         <f>B67+B68+B69+B70+B71+B72+B73+B74+B75</f>
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -21681,15 +21818,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -22022,15 +22159,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="253"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="263"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5"/>
@@ -22160,9 +22297,9 @@
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="254"/>
-      <c r="E10" s="254"/>
-      <c r="F10" s="254"/>
+      <c r="D10" s="264"/>
+      <c r="E10" s="264"/>
+      <c r="F10" s="264"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7">
@@ -22305,15 +22442,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="261" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>

</xml_diff>